<commit_message>
C6: bổ sung loại bằng chứng chất lượng/ESG vào backlog, kế hoạch module và plan
- Backlog C6: tách chứng nhận chất lượng thành loại có cấu trúc (ISO 9001/14001, HACCP, BRCGS, IFS, BSCI, WRAP, SMETA,
  CE marking, kết quả kiểm nghiệm lab), thêm certificate_number và issuer; danh sách loại do luật TM duyệt
- Backlog C6/X4: nhắc nộp hồ sơ EUDR cho mã cà phê nếu luật TM yêu cầu (chỉ nhắc, không loại tự động, không phải công cụ)
- C6 bật dòng evidence của điểm hoàn thiện B3 và thêm job nền hằng ngày tính lại điểm
- Chỉ sửa 4 chuỗi trong xlsx (sharedStrings), giữ nguyên mọi phần khác kể cả giá trị công thức đã tính
- Cập nhật KE_HOACH_CODE_THEO_MODULE.md (M6) và plan thực thi (Q6, Task 19)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/backlog/EVFTA_eu_Backlog_MVP.xlsx
+++ b/docs/backlog/EVFTA_eu_Backlog_MVP.xlsx
@@ -779,10 +779,10 @@
     <t xml:space="preserve">Bằng chứng xuất xứ + danh sách bắt buộc theo nhóm hàng</t>
   </si>
   <si>
-    <t xml:space="preserve">Bảng evidences: loại (chứng nhận chất lượng, EUR.1 đã cấp — che giá, tự chứng nhận xuất xứ lô ≤ 6.000 EUR, chứng nhận gạo thơm NĐ 103/2020, hồ sơ EUDR, giấy khai thác IUU), file, issued_at, expires_at (xuất xứ: +12 tháng), approval_status; danh sách bắt buộc theo nhóm hàng; 'EVFTA-verified' = verified + đủ bằng chứng bắt buộc còn hạn.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hồ sơ hiện danh sách kiểm theo nhóm hàng; bằng chứng hết hạn thì tự hạ mức.</t>
+    <t xml:space="preserve">Bảng evidences: loại (chứng nhận chất lượng, EUR.1 đã cấp — che giá, tự chứng nhận xuất xứ lô ≤ 6.000 EUR, chứng nhận gạo thơm NĐ 103/2020, hồ sơ EUDR, giấy khai thác IUU), file, issued_at, expires_at (xuất xứ: +12 tháng), approval_status; danh sách bắt buộc theo nhóm hàng; 'EVFTA-verified' = verified + đủ bằng chứng bắt buộc còn hạn. BỔ SUNG 29/09/2026 (theo nghiên cứu của PO; danh sách loại do luật TM duyệt trước khi nhập): (1) tách 'chứng nhận chất lượng' thành các loại có cấu trúc — hệ thống quản lý: ISO 9001, ISO 14001, HACCP, BRCGS, IFS; trách nhiệm xã hội: BSCI, WRAP, SMETA; kỹ thuật: CE marking; kết quả kiểm nghiệm của phòng lab (ghi tên phòng lab và số hiệu báo cáo); (2) lưu thêm certificate_number và issuer để đối chiếu với tổ chức cấp; (3) loại nào bắt buộc theo nhóm hàng do luật TM nhập vào required_evidence_rules, không viết cứng trong code; (4) nếu luật TM yêu cầu, với mã cà phê 0901.11 và 0901.21 nhắc nộp hồ sơ EUDR (chỉ nhắc, không loại tự động, không phải công cụ EUDR — xem X4); (5) bật dòng 'evidence' của điểm hoàn thiện B3 (completeness_weights.is_enabled), đếm bằng chứng đã nộp còn hạn, và thêm job nền tính lại điểm hoàn thiện hằng ngày (bằng chứng hết hạn không phát sự kiện) — gộp vào job quét hết hạn của I7.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hồ sơ hiện danh sách kiểm theo nhóm hàng; bằng chứng hết hạn thì tự hạ mức. Bổ sung: danh sách loại bằng chứng và nhóm hàng bắt buộc đã được luật TM duyệt; bằng chứng hết hạn thì điểm hoàn thiện giảm sau lần quét hằng ngày kế tiếp; không tính năng nào tự loại doanh nghiệp vì thiếu bằng chứng (chỉ verification.decide() đổi trạng thái xác minh).</t>
   </si>
   <si>
     <t xml:space="preserve">T5–6</t>
@@ -1406,7 +1406,7 @@
     <t xml:space="preserve">Công cụ ESG / CSRD / EUDR</t>
   </si>
   <si>
-    <t xml:space="preserve">Không làm công cụ; chỉ nhận hồ sơ EUDR như một loại bằng chứng (C6).</t>
+    <t xml:space="preserve">Không làm công cụ; chỉ nhận hồ sơ EUDR như một loại bằng chứng (C6). Nhắc nộp hồ sơ EUDR cho mã cà phê (nếu luật TM yêu cầu) thuộc C6, không phải công cụ. Không làm điểm 'loại ngay' (knockout) — xem docs/roadmap/2026-09-29-nghien-cuu-trong-so-uy-tin.md.</t>
   </si>
   <si>
     <t xml:space="preserve">VYBE X7</t>
@@ -1559,7 +1559,7 @@
     <t xml:space="preserve">verification_requests, verification_decisions, evidences</t>
   </si>
   <si>
-    <t xml:space="preserve">request: company_id, submitted_evidence_ids, status, submitted_at · decision: reviewer_id, decision, reason, decided_at · evidence: type, file, issued_at, expires_at, approval_status</t>
+    <t xml:space="preserve">request: company_id, submitted_evidence_ids, status, submitted_at · decision: reviewer_id, decision, reason, decided_at · evidence: type, file, certificate_number, issuer, issued_at, expires_at, approval_status</t>
   </si>
   <si>
     <t xml:space="preserve">Lý do bắt buộc khi từ chối/yêu cầu bổ sung; bằng chứng xuất xứ hạn 12 tháng</t>

</xml_diff>